<commit_message>
Catalog: pick the canonical rarity, not the displayed-printing one
The card detail page lists 'Rarity' twice — once for the printing the page
defaults to (which is 'showcase' for cards whose default view is the alt-art)
and once for the underlying card. parse_card_detail returned both in
fields['rarity'], and we were taking [0] (the printing-specific one), so 59
cards came out labeled 'showcase' that are actually rare/epic/common
underneath.

Fixed at the source (fetch_card_catalog + the two metadata-fetch loops in
main + update_archetype): drop 'showcase' entries first, then take the
first remaining rarity.

Targeted re-fetch of only the 59 affected slugs (rather than the full 768)
flipped 51 to their real rarity — 31 rare, 17 epic, 3 common — and left 8
that genuinely are showcase. Propagated to all 40 legend cards_meta entries
(248 patched), regenerated collection-template.xlsx, staples.js, and every
data.js / cards.json downstream.
</commit_message>
<xml_diff>
--- a/collection-template.xlsx
+++ b/collection-template.xlsx
@@ -741,7 +741,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>common</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1957,7 +1957,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>epic</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2983,7 +2983,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -3363,7 +3363,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -3477,7 +3477,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>epic</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -3857,7 +3857,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>common</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -6631,7 +6631,7 @@
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>epic</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
@@ -6707,7 +6707,7 @@
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>epic</t>
         </is>
       </c>
       <c r="G165" t="inlineStr">
@@ -7961,7 +7961,7 @@
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G198" t="inlineStr">
@@ -8151,7 +8151,7 @@
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>epic</t>
         </is>
       </c>
       <c r="G203" t="inlineStr">
@@ -8607,7 +8607,7 @@
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>common</t>
         </is>
       </c>
       <c r="G215" t="inlineStr">
@@ -9519,7 +9519,7 @@
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G239" t="inlineStr">
@@ -9823,7 +9823,7 @@
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>epic</t>
         </is>
       </c>
       <c r="G247" t="inlineStr">
@@ -9861,7 +9861,7 @@
       </c>
       <c r="F248" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G248" t="inlineStr">
@@ -10013,7 +10013,7 @@
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G252" t="inlineStr">
@@ -10089,7 +10089,7 @@
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G254" t="inlineStr">
@@ -10165,7 +10165,7 @@
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G256" t="inlineStr">
@@ -10393,7 +10393,7 @@
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G262" t="inlineStr">
@@ -10469,7 +10469,7 @@
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G264" t="inlineStr">
@@ -13509,7 +13509,7 @@
       </c>
       <c r="F344" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G344" t="inlineStr">
@@ -14801,7 +14801,7 @@
       </c>
       <c r="F378" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G378" t="inlineStr">
@@ -15865,7 +15865,7 @@
       </c>
       <c r="F406" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G406" t="inlineStr">
@@ -16929,7 +16929,7 @@
       </c>
       <c r="F434" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G434" t="inlineStr">
@@ -17043,7 +17043,7 @@
       </c>
       <c r="F437" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G437" t="inlineStr">
@@ -17271,7 +17271,7 @@
       </c>
       <c r="F443" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>epic</t>
         </is>
       </c>
       <c r="G443" t="inlineStr">
@@ -18107,7 +18107,7 @@
       </c>
       <c r="F465" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G465" t="inlineStr">
@@ -18183,7 +18183,7 @@
       </c>
       <c r="F467" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G467" t="inlineStr">
@@ -18411,7 +18411,7 @@
       </c>
       <c r="F473" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>epic</t>
         </is>
       </c>
       <c r="G473" t="inlineStr">
@@ -19209,7 +19209,7 @@
       </c>
       <c r="F494" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G494" t="inlineStr">
@@ -19247,7 +19247,7 @@
       </c>
       <c r="F495" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G495" t="inlineStr">
@@ -19475,7 +19475,7 @@
       </c>
       <c r="F501" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>epic</t>
         </is>
       </c>
       <c r="G501" t="inlineStr">
@@ -19589,7 +19589,7 @@
       </c>
       <c r="F504" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>epic</t>
         </is>
       </c>
       <c r="G504" t="inlineStr">
@@ -19627,7 +19627,7 @@
       </c>
       <c r="F505" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G505" t="inlineStr">
@@ -20083,7 +20083,7 @@
       </c>
       <c r="F517" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G517" t="inlineStr">
@@ -20311,7 +20311,7 @@
       </c>
       <c r="F523" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G523" t="inlineStr">
@@ -21983,7 +21983,7 @@
       </c>
       <c r="F567" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G567" t="inlineStr">
@@ -22287,7 +22287,7 @@
       </c>
       <c r="F575" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>epic</t>
         </is>
       </c>
       <c r="G575" t="inlineStr">
@@ -23237,7 +23237,7 @@
       </c>
       <c r="F600" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G600" t="inlineStr">
@@ -23351,7 +23351,7 @@
       </c>
       <c r="F603" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>epic</t>
         </is>
       </c>
       <c r="G603" t="inlineStr">
@@ -24263,7 +24263,7 @@
       </c>
       <c r="F627" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G627" t="inlineStr">
@@ -24453,7 +24453,7 @@
       </c>
       <c r="F632" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>epic</t>
         </is>
       </c>
       <c r="G632" t="inlineStr">
@@ -24567,7 +24567,7 @@
       </c>
       <c r="F635" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>epic</t>
         </is>
       </c>
       <c r="G635" t="inlineStr">
@@ -25669,7 +25669,7 @@
       </c>
       <c r="F664" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>epic</t>
         </is>
       </c>
       <c r="G664" t="inlineStr">
@@ -26581,7 +26581,7 @@
       </c>
       <c r="F688" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G688" t="inlineStr">
@@ -26809,7 +26809,7 @@
       </c>
       <c r="F694" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>epic</t>
         </is>
       </c>
       <c r="G694" t="inlineStr">
@@ -26847,7 +26847,7 @@
       </c>
       <c r="F695" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>epic</t>
         </is>
       </c>
       <c r="G695" t="inlineStr">
@@ -27683,7 +27683,7 @@
       </c>
       <c r="F717" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G717" t="inlineStr">
@@ -27835,7 +27835,7 @@
       </c>
       <c r="F721" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G721" t="inlineStr">
@@ -28557,7 +28557,7 @@
       </c>
       <c r="F740" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G740" t="inlineStr">
@@ -28633,7 +28633,7 @@
       </c>
       <c r="F742" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G742" t="inlineStr">
@@ -28785,7 +28785,7 @@
       </c>
       <c r="F746" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G746" t="inlineStr">

</xml_diff>

<commit_message>
Collection xlsx: use full archetype name for legend cards
The riftdecks card detail page lists 'name: Scorn of the Moon' for the
legend printing rather than the canonical 'Diana, Scorn of the Moon',
so build_collection_template was emitting just the epithet. Pull the
full archetype name from champions.js when the card type is legend so
the xlsx is identifiable and matches TCGplayer-style names that paste
the comma form.
</commit_message>
<xml_diff>
--- a/collection-template.xlsx
+++ b/collection-template.xlsx
@@ -9841,7 +9841,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>Daughter of the Void</t>
+          <t>Kai'sa, Daughter of the Void</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
@@ -9917,7 +9917,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>Relentless Storm</t>
+          <t>Volibear, Relentless Storm</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
@@ -9993,7 +9993,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>Loose Cannon</t>
+          <t>Jinx, Loose Cannon</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
@@ -10069,7 +10069,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>Hand of Noxus</t>
+          <t>Darius, Hand of Noxus</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
@@ -10145,7 +10145,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>Nine-Tailed Fox</t>
+          <t>Ahri, Nine-Tailed Fox</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -10221,7 +10221,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>Blind Monk</t>
+          <t>Lee Sin, Blind Monk</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
@@ -10297,7 +10297,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>Unforgiven</t>
+          <t>Yasuo, Unforgiven</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
@@ -10373,7 +10373,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>Radiant Dawn</t>
+          <t>Leona, Radiant Dawn</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
@@ -10449,7 +10449,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>Swift Scout</t>
+          <t>Teemo, Swift Scout</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
@@ -10525,7 +10525,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>Herald of the Arcane</t>
+          <t>Viktor, Herald of the Arcane</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
@@ -10601,7 +10601,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>Bounty Hunter</t>
+          <t>Miss Fortune, Bounty Hunter</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
@@ -10677,7 +10677,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>The Boss</t>
+          <t>Sett, The Boss</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
@@ -12463,7 +12463,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Dark Child - Starter</t>
+          <t>Annie, Dark Child</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -12539,7 +12539,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Wuju Bladesman - Starter</t>
+          <t>Master Yi, Wuju Bladesman</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -12615,7 +12615,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Lady of Luminosity - Starter</t>
+          <t>Lux, Lady of Luminosity</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -12691,7 +12691,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Might of Demacia - Starter</t>
+          <t>Garen, Might of Demacia</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -19607,7 +19607,7 @@
       </c>
       <c r="B505" t="inlineStr">
         <is>
-          <t>Mechanized Menace</t>
+          <t>Rumble, Mechanized Menace</t>
         </is>
       </c>
       <c r="C505" t="inlineStr">
@@ -19683,7 +19683,7 @@
       </c>
       <c r="B507" t="inlineStr">
         <is>
-          <t>Purifier</t>
+          <t>Lucian, Purifier</t>
         </is>
       </c>
       <c r="C507" t="inlineStr">
@@ -19759,7 +19759,7 @@
       </c>
       <c r="B509" t="inlineStr">
         <is>
-          <t>Glorious Executioner</t>
+          <t>Draven, Glorious Executioner</t>
         </is>
       </c>
       <c r="C509" t="inlineStr">
@@ -19835,7 +19835,7 @@
       </c>
       <c r="B511" t="inlineStr">
         <is>
-          <t>Void Burrower</t>
+          <t>Reksai, Void Burrower</t>
         </is>
       </c>
       <c r="C511" t="inlineStr">
@@ -19911,7 +19911,7 @@
       </c>
       <c r="B513" t="inlineStr">
         <is>
-          <t>Fire Below the Mountain</t>
+          <t>Ornn, Fire Below the Mountain</t>
         </is>
       </c>
       <c r="C513" t="inlineStr">
@@ -20063,7 +20063,7 @@
       </c>
       <c r="B517" t="inlineStr">
         <is>
-          <t>Grandmaster at Arms</t>
+          <t>Jax, Grandmaster at Arms</t>
         </is>
       </c>
       <c r="C517" t="inlineStr">
@@ -20139,7 +20139,7 @@
       </c>
       <c r="B519" t="inlineStr">
         <is>
-          <t>Blade Dancer</t>
+          <t>Irelia, Blade Dancer</t>
         </is>
       </c>
       <c r="C519" t="inlineStr">
@@ -20215,7 +20215,7 @@
       </c>
       <c r="B521" t="inlineStr">
         <is>
-          <t>Emperor of the Sands</t>
+          <t>Azir, Emperor of the Sands</t>
         </is>
       </c>
       <c r="C521" t="inlineStr">
@@ -20291,7 +20291,7 @@
       </c>
       <c r="B523" t="inlineStr">
         <is>
-          <t>Prodigal Explorer</t>
+          <t>Ezreal, Prodigal Explorer</t>
         </is>
       </c>
       <c r="C523" t="inlineStr">
@@ -20367,7 +20367,7 @@
       </c>
       <c r="B525" t="inlineStr">
         <is>
-          <t>Chem-Baroness</t>
+          <t>Renata Glasc, Chem-Baroness</t>
         </is>
       </c>
       <c r="C525" t="inlineStr">
@@ -20443,7 +20443,7 @@
       </c>
       <c r="B527" t="inlineStr">
         <is>
-          <t>Battle Mistress</t>
+          <t>Sivir, Battle Mistress</t>
         </is>
       </c>
       <c r="C527" t="inlineStr">
@@ -20519,7 +20519,7 @@
       </c>
       <c r="B529" t="inlineStr">
         <is>
-          <t>Grand Duelist</t>
+          <t>Fiora, Grand Duelist</t>
         </is>
       </c>
       <c r="C529" t="inlineStr">
@@ -28005,7 +28005,7 @@
       </c>
       <c r="B726" t="inlineStr">
         <is>
-          <t>Virtuoso</t>
+          <t>Jhin, Virtuoso</t>
         </is>
       </c>
       <c r="C726" t="inlineStr">
@@ -28081,7 +28081,7 @@
       </c>
       <c r="B728" t="inlineStr">
         <is>
-          <t>Pridestalker</t>
+          <t>Rengar, Pridestalker</t>
         </is>
       </c>
       <c r="C728" t="inlineStr">
@@ -28157,7 +28157,7 @@
       </c>
       <c r="B730" t="inlineStr">
         <is>
-          <t>Bloodharbor Ripper</t>
+          <t>Pyke, Bloodharbor Ripper</t>
         </is>
       </c>
       <c r="C730" t="inlineStr">
@@ -28233,7 +28233,7 @@
       </c>
       <c r="B732" t="inlineStr">
         <is>
-          <t>Piltover Enforcer</t>
+          <t>Vi, Piltover Enforcer</t>
         </is>
       </c>
       <c r="C732" t="inlineStr">
@@ -28309,7 +28309,7 @@
       </c>
       <c r="B734" t="inlineStr">
         <is>
-          <t>Bashful Bloom</t>
+          <t>Lillia, Bashful Bloom</t>
         </is>
       </c>
       <c r="C734" t="inlineStr">
@@ -28385,7 +28385,7 @@
       </c>
       <c r="B736" t="inlineStr">
         <is>
-          <t>Wuju Master</t>
+          <t>Master Yi, Wuju Master</t>
         </is>
       </c>
       <c r="C736" t="inlineStr">
@@ -28461,7 +28461,7 @@
       </c>
       <c r="B738" t="inlineStr">
         <is>
-          <t>Gloomist</t>
+          <t>Vex, Gloomist</t>
         </is>
       </c>
       <c r="C738" t="inlineStr">
@@ -28537,7 +28537,7 @@
       </c>
       <c r="B740" t="inlineStr">
         <is>
-          <t>Green Father</t>
+          <t>Ivern, Green Father</t>
         </is>
       </c>
       <c r="C740" t="inlineStr">
@@ -28613,7 +28613,7 @@
       </c>
       <c r="B742" t="inlineStr">
         <is>
-          <t>Scorn of the Moon</t>
+          <t>Diana, Scorn of the Moon</t>
         </is>
       </c>
       <c r="C742" t="inlineStr">
@@ -28689,7 +28689,7 @@
       </c>
       <c r="B744" t="inlineStr">
         <is>
-          <t>Deceiver</t>
+          <t>Leblanc, Deceiver</t>
         </is>
       </c>
       <c r="C744" t="inlineStr">
@@ -28765,7 +28765,7 @@
       </c>
       <c r="B746" t="inlineStr">
         <is>
-          <t>Voidreaver</t>
+          <t>Khazix, Voidreaver</t>
         </is>
       </c>
       <c r="C746" t="inlineStr">
@@ -28841,7 +28841,7 @@
       </c>
       <c r="B748" t="inlineStr">
         <is>
-          <t>Keeper of the Hammer</t>
+          <t>Poppy, Keeper of the Hammer</t>
         </is>
       </c>
       <c r="C748" t="inlineStr">

</xml_diff>

<commit_message>
Catalog: walk variant URLs when main page is showcase-only
A handful of cards (Irelia Fervent, Sett the Boss, Lillia BB, MF, Viktor,
Volibear, Soraka, Aphelios) only show showcase rarity on their default
detail page even though a standard-rarity printing exists. The variant
URLs /cards/<slug>/<printing-id> render the per-printing rarity, so
fetch_card_catalog now follows them and picks the first non-showcase
rarity it finds.

Showcase is always optional alt-art — for closeness/cart scoring we
weight by the underlying buyable rarity, not the showcase tier. Targeted
re-fetch updated all 8 cards (7 rare, 1 epic) and propagated to 25
per-legend rarity entries across 19 legends.
</commit_message>
<xml_diff>
--- a/collection-template.xlsx
+++ b/collection-template.xlsx
@@ -9937,7 +9937,7 @@
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G250" t="inlineStr">
@@ -10545,7 +10545,7 @@
       </c>
       <c r="F266" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G266" t="inlineStr">
@@ -10621,7 +10621,7 @@
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G268" t="inlineStr">
@@ -10697,7 +10697,7 @@
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G270" t="inlineStr">
@@ -14611,7 +14611,7 @@
       </c>
       <c r="F373" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G373" t="inlineStr">
@@ -14915,7 +14915,7 @@
       </c>
       <c r="F381" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>epic</t>
         </is>
       </c>
       <c r="G381" t="inlineStr">
@@ -19323,7 +19323,7 @@
       </c>
       <c r="F497" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G497" t="inlineStr">
@@ -28329,7 +28329,7 @@
       </c>
       <c r="F734" t="inlineStr">
         <is>
-          <t>showcase</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="G734" t="inlineStr">

</xml_diff>